<commit_message>
Update reference Excel files for income transaction type feature
Regenerate all reference Excel files to include the new is_income field
in entries and allocations sheets. All Excel files now have 11 columns
in the entries sheet (added is_income column).

All tests now pass (25/25).

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,11 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>is_income</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>category</t>
         </is>
       </c>
@@ -574,7 +579,10 @@
       <c r="J2" t="b">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>FOOD</t>
         </is>
@@ -591,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,25 +630,30 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>is_income</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>original_share</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>original_currency</t>
         </is>
@@ -669,23 +682,26 @@
       <c r="F2" t="b">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>15</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>15</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
Rename split_view to transaction_ledger and use snake_case columns
- Rename sheet from split_view to transaction_ledger for clarity
- Change all column names to snake_case (date, description, category, type, cost, currency) to match other sheets
- Fix date sorting to use datetime objects before formatting to strings
- Add comprehensive test covering expense, reimbursement, income, and non-participating members
- Update all 8 reference Excel files with transaction_ledger sheet

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -12,6 +12,7 @@
     <sheet name="allocations" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="attachments" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="balances" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="transaction_ledger" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -788,4 +789,91 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Receipt</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FOOD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>